<commit_message>
File cleanup, start year calibration, and update to data source for coal/lignite fuel price split
</commit_message>
<xml_diff>
--- a/InputData/elec/HYECFCA/HIst Year Elec Cap Fac Cal Adjust.xlsx
+++ b/InputData/elec/HYECFCA/HIst Year Elec Cap Fac Cal Adjust.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\HYECFCA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\HYECFCA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818123C5-1164-4CA3-91CD-278A2968B27A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DE4846-ACEE-4A36-8C8F-2120F7B91DAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1830" windowWidth="43200" windowHeight="17025" xr2:uid="{2434D2BD-6D34-4476-A32C-19CE7C594793}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{2434D2BD-6D34-4476-A32C-19CE7C594793}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="HYECFCA" sheetId="2" r:id="rId2"/>
+    <sheet name="Calibration 2025" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>HYECFCA Historical Year Electricity Capacity Factor Calibration Adjustment</t>
   </si>
@@ -48,9 +49,6 @@
     <t>Sources:</t>
   </si>
   <si>
-    <t>(n/a)</t>
-  </si>
-  <si>
     <t>hydrogen combined cycle es</t>
   </si>
   <si>
@@ -127,6 +125,60 @@
   </si>
   <si>
     <t>multiplier (dmnl, %)</t>
+  </si>
+  <si>
+    <t>2025 HYECFCA calibration: multiplier = EIA 2025 observed net generation / model 2025 generation at HYECFCA = 1</t>
+  </si>
+  <si>
+    <t>Applies to SYSHECF-gated sources only (BDTPTUMCF = 0). MCF-gated sources (coal, gas, oil, CCS, H2) stay at 1 - their generation is set by economic dispatch, not capacity factors. 2026+ stays at 1 so the forecast is untouched. One iteration sufficed: the follow-up run reproduced every EIA value to &lt;0.005%.</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>EIA 2025 net generation (MWh)</t>
+  </si>
+  <si>
+    <t>HYECFCA 2025</t>
+  </si>
+  <si>
+    <t>nuclear</t>
+  </si>
+  <si>
+    <t>hydro</t>
+  </si>
+  <si>
+    <t>onshore wind</t>
+  </si>
+  <si>
+    <t>solar PV</t>
+  </si>
+  <si>
+    <t>solar thermal</t>
+  </si>
+  <si>
+    <t>biomass</t>
+  </si>
+  <si>
+    <t>geothermal</t>
+  </si>
+  <si>
+    <t>offshore wind</t>
+  </si>
+  <si>
+    <t>municipal solid waste</t>
+  </si>
+  <si>
+    <t>EIA source: EIA-923 2025 Early Release (30JUN2026 file), Page 1 Generation and Fuel Data, bucketed to EPS sources per the BGDPbES workbook fuel/prime-mover lookups and sector filters (Electric Utility + NAICS-22; industrial/commercial CHP excluded). The identical pasted dataset and SUMIFS live in the SYSHECF workbook's '923' tab (InputData/elec/SYSHECF) - its per-source sums reproduce column B exactly.</t>
+  </si>
+  <si>
+    <t>Model run: eps-us develop_4.0.6, BAU (no .cin), run CAL25H0 2026-09-10 - HEAD 894015da plus the uncommitted 2026-09-10 SYSHECF calibration (biomass/MSW/peaker/petroleum tied to EIA 2025 CFs). Model 2025 gen values pasted from CAL25H0.tab (BAU Electricity Generation by Type). Re-derive by re-running BAU with HYECFCA set to 1.</t>
+  </si>
+  <si>
+    <t>2025: EIA-923 2025 Early Release net generation vs model run at HYECFCA=1 - see 'Calibration 2025' tab (added 2026-09-10). All other years: 1 (no adjustment).</t>
+  </si>
+  <si>
+    <t>Model 2025 generation, HYECFCA=1 (MWh, from CAL25H0.tab - Vensim exports 6 significant figures)</t>
   </si>
 </sst>
 </file>
@@ -520,7 +572,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -542,7 +594,7 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1">
         <v>2025</v>
@@ -625,7 +677,7 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -708,7 +760,7 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -791,7 +843,7 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -874,10 +926,11 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <f>'Calibration 2025'!D5</f>
+        <v>0.99925866186869106</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -957,10 +1010,11 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <f>'Calibration 2025'!D6</f>
+        <v>0.97656769537997867</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1040,10 +1094,11 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <f>'Calibration 2025'!D7</f>
+        <v>0.99049996775136739</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -1123,10 +1178,11 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <f>'Calibration 2025'!D8</f>
+        <v>1.0669161325664203</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1206,10 +1262,11 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <f>'Calibration 2025'!D9</f>
+        <v>0.93648670812995327</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1289,10 +1346,11 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <f>'Calibration 2025'!D10</f>
+        <v>1.0238947796972699</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1372,10 +1430,11 @@
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <f>'Calibration 2025'!D11</f>
+        <v>1.0049882422482364</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1455,7 +1514,7 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1538,7 +1597,7 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1621,7 +1680,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1704,10 +1763,11 @@
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <f>'Calibration 2025'!D12</f>
+        <v>1.0687524097695031</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1787,7 +1847,7 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1870,7 +1930,7 @@
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1953,10 +2013,11 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <f>'Calibration 2025'!D13</f>
+        <v>0.99999935568255771</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -2036,7 +2097,7 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -2119,7 +2180,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -2202,7 +2263,7 @@
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -2285,7 +2346,7 @@
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -2368,7 +2429,7 @@
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23">
         <v>1</v>
@@ -2451,7 +2512,7 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -2534,7 +2595,7 @@
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B25">
         <v>1</v>
@@ -2617,7 +2678,7 @@
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -2696,6 +2757,185 @@
       </c>
       <c r="AA26">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0F07B30-2289-4DFA-B2A9-691D5E6D350E}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5">
+        <v>785304392</v>
+      </c>
+      <c r="C5">
+        <v>785887000</v>
+      </c>
+      <c r="D5">
+        <f t="shared" ref="D5:D13" si="0">B5/C5</f>
+        <v>0.99925866186869106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6">
+        <v>239131155</v>
+      </c>
+      <c r="C6">
+        <v>244869000</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>0.97656769537997867</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7">
+        <v>460717193</v>
+      </c>
+      <c r="C7">
+        <v>465136000</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>0.99049996775136739</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8">
+        <v>292148310</v>
+      </c>
+      <c r="C8">
+        <v>273825000</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>1.0669161325664203</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9">
+        <v>2854861</v>
+      </c>
+      <c r="C9">
+        <v>3048480</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>0.93648670812995327</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10">
+        <v>16850134</v>
+      </c>
+      <c r="C10">
+        <v>16456900</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>1.0238947796972699</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11">
+        <v>15641838</v>
+      </c>
+      <c r="C11">
+        <v>15564200</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>1.0049882422482364</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12">
+        <v>673578</v>
+      </c>
+      <c r="C12">
+        <v>630247</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>1.0687524097695031</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13">
+        <v>6208116</v>
+      </c>
+      <c r="C13">
+        <v>6208120</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>0.99999935568255771</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>